<commit_message>
fix wrong correct_key column in practice trials retrieval and add more explanations for retrieval trials to practice task
</commit_message>
<xml_diff>
--- a/sequences/retr_trials_prc.xlsx
+++ b/sequences/retr_trials_prc.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="37">
   <si>
     <t>trial_type</t>
   </si>
@@ -82,9 +82,6 @@
   </si>
   <si>
     <t>distance_correct</t>
-  </si>
-  <si>
-    <t>up</t>
   </si>
   <si>
     <t>image_dur_retr</t>
@@ -526,22 +523,22 @@
         <v>18</v>
       </c>
       <c r="J1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M1" t="s">
+        <v>23</v>
+      </c>
+      <c r="N1" t="s">
         <v>21</v>
       </c>
-      <c r="L1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M1" t="s">
-        <v>24</v>
-      </c>
-      <c r="N1" t="s">
-        <v>22</v>
-      </c>
       <c r="O1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -576,7 +573,7 @@
         <v>0.5</v>
       </c>
       <c r="L2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M2">
         <v>0.45</v>
@@ -585,7 +582,7 @@
         <v>1.95</v>
       </c>
       <c r="O2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
@@ -620,7 +617,7 @@
         <v>0.5</v>
       </c>
       <c r="L3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="M3">
         <v>0.52</v>
@@ -629,7 +626,7 @@
         <v>1.89</v>
       </c>
       <c r="O3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
@@ -652,7 +649,7 @@
         <v>11</v>
       </c>
       <c r="H4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="I4">
         <v>3</v>
@@ -664,7 +661,7 @@
         <v>0.5</v>
       </c>
       <c r="L4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M4">
         <v>0.61</v>
@@ -673,7 +670,7 @@
         <v>2.15</v>
       </c>
       <c r="O4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
@@ -696,7 +693,7 @@
         <v>11</v>
       </c>
       <c r="H5" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I5">
         <v>2</v>
@@ -708,7 +705,7 @@
         <v>0.5</v>
       </c>
       <c r="L5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M5">
         <v>0.45</v>
@@ -717,7 +714,7 @@
         <v>1.95</v>
       </c>
       <c r="O5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
@@ -752,7 +749,7 @@
         <v>0.5</v>
       </c>
       <c r="L6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="M6">
         <v>0.52</v>
@@ -761,7 +758,7 @@
         <v>1.89</v>
       </c>
       <c r="O6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
@@ -772,7 +769,7 @@
         <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
@@ -784,7 +781,7 @@
         <v>8</v>
       </c>
       <c r="H7" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="I7">
         <v>4</v>
@@ -796,7 +793,7 @@
         <v>0.5</v>
       </c>
       <c r="L7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M7">
         <v>0.61</v>
@@ -805,7 +802,7 @@
         <v>2.15</v>
       </c>
       <c r="O7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
@@ -828,7 +825,7 @@
         <v>8</v>
       </c>
       <c r="H8" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="I8">
         <v>3</v>
@@ -840,7 +837,7 @@
         <v>0.5</v>
       </c>
       <c r="L8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="M8">
         <v>0.52</v>
@@ -849,7 +846,7 @@
         <v>1.89</v>
       </c>
       <c r="O8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
@@ -872,7 +869,7 @@
         <v>8</v>
       </c>
       <c r="H9" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="I9">
         <v>2</v>
@@ -884,7 +881,7 @@
         <v>0.5</v>
       </c>
       <c r="L9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M9">
         <v>0.61</v>
@@ -893,7 +890,7 @@
         <v>2.15</v>
       </c>
       <c r="O9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>